<commit_message>
Templates: add Opening/Closing Balance, Net Cash Flow with formulas
Both templates now include:
- Opening Balance row at top (enter manually for first month)
- TOTAL INFLOW / TOTAL OUTFLOW with SUM formulas
- NET CASH FLOW = Total Inflow - Total Outflow
- CLOSING BALANCE = Opening + Net Cash Flow

Each month's closing should carry forward as next month's opening,
giving a built-in sanity check on the figures.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/cash-flow-forecast-imperial.xlsx
+++ b/public/cash-flow-forecast-imperial.xlsx
@@ -399,9 +399,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G20"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
@@ -435,58 +435,40 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CASH INFLOW</v>
+        <v>OPENING BALANCE</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Gross Sales - Retail</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Gross Sales - Online</v>
-      </c>
-      <c r="B4">
-        <v>0</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
+        <v>CASH INFLOW</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Other Income</v>
+        <v>Gross Sales - Retail</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -509,7 +491,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>TOTAL INFLOW</v>
+        <v>Gross Sales - Online</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -532,63 +514,69 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>Other Income</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>CASH OUTFLOW</v>
+        <v>TOTAL INFLOW</v>
+      </c>
+      <c r="B8">
+        <f>SUM(B5:B7)</f>
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <f>SUM(C5:C7)</f>
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <f>SUM(D5:D7)</f>
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <f>SUM(E5:E7)</f>
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <f>SUM(F5:F7)</f>
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <f>SUM(G5:G7)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Salaries</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Marketing</v>
-      </c>
-      <c r="B10">
-        <v>0</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
+        <v>CASH OUTFLOW</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Admin Expenses</v>
+        <v>Salaries</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -611,7 +599,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Less: Depreciation (non-cash)</v>
+        <v>Marketing</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -634,7 +622,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>TOTAL OUTFLOW</v>
+        <v>Admin Expenses</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -657,35 +645,132 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v/>
+        <v>Less: Depreciation (non-cash)</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
+        <v>TOTAL OUTFLOW</v>
+      </c>
+      <c r="B15">
+        <f>SUM(B11:B14)</f>
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <f>SUM(C11:C14)</f>
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <f>SUM(D11:D14)</f>
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <f>SUM(E11:E14)</f>
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <f>SUM(F11:F14)</f>
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <f>SUM(G11:G14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>NET CASH FLOW</v>
+      </c>
+      <c r="B17">
+        <f>B8-B15</f>
+        <v>0</v>
+      </c>
+      <c r="C17">
+        <f>C8-C15</f>
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <f>D8-D15</f>
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <f>E8-E15</f>
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <f>F8-F15</f>
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <f>G8-G15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
         <v>CLOSING BALANCE</v>
       </c>
-      <c r="B15">
-        <v>0</v>
-      </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15">
-        <v>0</v>
+      <c r="B18">
+        <f>B2+B17</f>
+        <v>0</v>
+      </c>
+      <c r="C18">
+        <f>C2+C17</f>
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <f>D2+D17</f>
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <f>E2+E17</f>
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <f>F2+F17</f>
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <f>G2+G17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Note: Each month closing should equal next month opening. Depreciation is included as outflow but represents non-cash — net cash flow reflects actual cash movement.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: forecast not showing — templates now start from June 2026
Three fixes:
1. Templates now include June 2026 (current month) through Dec 2026.
   Previously started from July, so uploads had no data for this month.
2. Executive page now shows the nearest available forecast month if
   current month has no data — won't show blank anymore.
3. Fixed quarterly_forecasts using hardcoded Unze Trading ID instead
   of the actual company ID — Imperial uploads now save correctly.

Re-upload the forecast for both companies using the updated templates.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/cash-flow-forecast-imperial.xlsx
+++ b/public/cash-flow-forecast-imperial.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:H20"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -408,6 +408,7 @@
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -415,21 +416,24 @@
         <v/>
       </c>
       <c r="B1" s="1">
+        <v>46174</v>
+      </c>
+      <c r="C1" s="1">
         <v>46204</v>
       </c>
-      <c r="C1" s="1">
+      <c r="D1" s="1">
         <v>46235</v>
       </c>
-      <c r="D1" s="1">
+      <c r="E1" s="1">
         <v>46266</v>
       </c>
-      <c r="E1" s="1">
+      <c r="F1" s="1">
         <v>46296</v>
       </c>
-      <c r="F1" s="1">
+      <c r="G1" s="1">
         <v>46327</v>
       </c>
-      <c r="G1" s="1">
+      <c r="H1" s="1">
         <v>46357</v>
       </c>
     </row>
@@ -455,6 +459,9 @@
       <c r="G2">
         <v>0</v>
       </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -488,6 +495,9 @@
       <c r="G5">
         <v>0</v>
       </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -511,6 +521,9 @@
       <c r="G6">
         <v>0</v>
       </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -534,6 +547,9 @@
       <c r="G7">
         <v>0</v>
       </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -563,6 +579,10 @@
         <f>SUM(G5:G7)</f>
         <v>0</v>
       </c>
+      <c r="H8">
+        <f>SUM(H5:H7)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -596,6 +616,9 @@
       <c r="G11">
         <v>0</v>
       </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -619,6 +642,9 @@
       <c r="G12">
         <v>0</v>
       </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -642,6 +668,9 @@
       <c r="G13">
         <v>0</v>
       </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -665,6 +694,9 @@
       <c r="G14">
         <v>0</v>
       </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -694,6 +726,10 @@
         <f>SUM(G11:G14)</f>
         <v>0</v>
       </c>
+      <c r="H15">
+        <f>SUM(H11:H14)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -728,6 +764,10 @@
         <f>G8-G15</f>
         <v>0</v>
       </c>
+      <c r="H17">
+        <f>H8-H15</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -757,6 +797,10 @@
         <f>G2+G17</f>
         <v>0</v>
       </c>
+      <c r="H18">
+        <f>H2+H17</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -765,12 +809,12 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Note: Each month closing should equal next month opening. Depreciation is included as outflow but represents non-cash — net cash flow reflects actual cash movement.</v>
+        <v>Note: Each month closing should equal next month opening. Depreciation is included as outflow but represents non-cash.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>